<commit_message>
standariser l interface des gestion des encoours dans le contexte du rapprochement
</commit_message>
<xml_diff>
--- a/gBanque/src/main/resources/nature_lignes_fonctionnelles.xlsx
+++ b/gBanque/src/main/resources/nature_lignes_fonctionnelles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hp\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{842F3AC5-12D1-4E06-8AC2-4E317D02529A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82444F85-1B90-459E-8C52-1FF15DDB8791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{BE083332-C395-4A21-9ECE-C8A5058013E8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>Label</t>
   </si>
@@ -102,6 +102,18 @@
   </si>
   <si>
     <t>Opération par laquelle une banque accorde un nouveau prêt pour rembourser un prêt existant, souvent dans des conditions plus favorables.</t>
+  </si>
+  <si>
+    <t>Préfinancement</t>
+  </si>
+  <si>
+    <t>C’est une ligne de crédit ou une avance de fonds accordée par une banque ou une institution financière afin de couvrir les besoins de trésorerie avant la réalisation effective des recettes.</t>
+  </si>
+  <si>
+    <t>Droit constaté</t>
+  </si>
+  <si>
+    <t>Elle concerne les créances ou recettes qui sont acquises et juridiquement exigibles, mais pas encore encaissées.</t>
   </si>
 </sst>
 </file>
@@ -473,7 +485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE120570-CC4C-49B1-A416-8811F4D69E4E}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.140625" customWidth="1"/>
@@ -568,6 +580,22 @@
         <v>21</v>
       </c>
     </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>